<commit_message>
Add full engineering workbook for DC-DC converter design
Uploaded the complete Excel-based engineering model for the 2.5 MW bidirectional DC-DC converter.

The workbook includes:
- System assumptions and operating conditions
- Power and current calculations
- Detailed loss breakdown (conduction, switching, magnetics, auxiliary)
- Efficiency analysis across load range
- Magnetics design assumptions and losses
- Semiconductor selection and loss estimates
- Thermal constraints and cooling considerations
- Control modes (CC, CV, CP) and phase-shift control
- Requirement compliance verification

This file serves as the primary technical backbone supporting all reported results and design decisions in the project.
</commit_message>
<xml_diff>
--- a/calculations/BESS_DC_DC_Converter_Efficiency_Model.xlsx
+++ b/calculations/BESS_DC_DC_Converter_Efficiency_Model.xlsx
@@ -5,15 +5,25 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reine\Desktop\Word for Hackathon\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\reine\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6979E59F-77BD-460C-A2D3-CAD782297788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{820F9BD2-D177-49AF-A6F9-02200529832E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66BDF9AC-B571-499F-BDD4-D641B197A894}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="10" xr2:uid="{66BDF9AC-B571-499F-BDD4-D641B197A894}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Assumptions" sheetId="2" r:id="rId2"/>
+    <sheet name="Power_Current" sheetId="3" r:id="rId3"/>
+    <sheet name="Loss_Breakdown" sheetId="4" r:id="rId4"/>
+    <sheet name="Efficiency" sheetId="5" r:id="rId5"/>
+    <sheet name="Magnetics" sheetId="6" r:id="rId6"/>
+    <sheet name="Semiconductors" sheetId="7" r:id="rId7"/>
+    <sheet name="Thermal_Constraints" sheetId="8" r:id="rId8"/>
+    <sheet name="Control_Modes" sheetId="9" r:id="rId9"/>
+    <sheet name="Requirement_Check" sheetId="10" r:id="rId10"/>
+    <sheet name="Fault_Handling" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="241">
   <si>
     <t>SECTION</t>
   </si>
@@ -129,16 +139,650 @@
   </si>
   <si>
     <t>A</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Bus</t>
+  </si>
+  <si>
+    <t>HVDC Bus Nominal Voltage</t>
+  </si>
+  <si>
+    <t>HVDC Bus Operating Min</t>
+  </si>
+  <si>
+    <t>HVDC Bus Operating Max</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Battery Nominal Voltage</t>
+  </si>
+  <si>
+    <t>Battery Operating Min</t>
+  </si>
+  <si>
+    <t>Battery Operating Max</t>
+  </si>
+  <si>
+    <t>Battery Energy Capacity</t>
+  </si>
+  <si>
+    <t>MWh</t>
+  </si>
+  <si>
+    <t>Power</t>
+  </si>
+  <si>
+    <t>Total Rated Power</t>
+  </si>
+  <si>
+    <t>Module Count</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Topology</t>
+  </si>
+  <si>
+    <t>Converter Topology</t>
+  </si>
+  <si>
+    <t>Dual Active Bridge</t>
+  </si>
+  <si>
+    <t>Isolation Method</t>
+  </si>
+  <si>
+    <t>High-Frequency Transformer</t>
+  </si>
+  <si>
+    <t>Devices</t>
+  </si>
+  <si>
+    <t>Semiconductor Technology</t>
+  </si>
+  <si>
+    <t>SiC MOSFET</t>
+  </si>
+  <si>
+    <t>Switching</t>
+  </si>
+  <si>
+    <t>Switching Frequency</t>
+  </si>
+  <si>
+    <t>Hz</t>
+  </si>
+  <si>
+    <t>Cooling</t>
+  </si>
+  <si>
+    <t>Cooling Method</t>
+  </si>
+  <si>
+    <t>Liquid Cooling</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>Ambient Temperature</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Efficiency at 100% load</t>
+  </si>
+  <si>
+    <t>&gt;=99.5%</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Efficiency at 50-100% load</t>
+  </si>
+  <si>
+    <t>&gt;=99.0%</t>
+  </si>
+  <si>
+    <t>Efficiency at 25-50% load</t>
+  </si>
+  <si>
+    <t>&gt;=98.5%</t>
+  </si>
+  <si>
+    <t>Max Junction Temperature</t>
+  </si>
+  <si>
+    <t>&lt;=125</t>
+  </si>
+  <si>
+    <t>Max Magnetics Hotspot</t>
+  </si>
+  <si>
+    <t>&lt;=120</t>
+  </si>
+  <si>
+    <t>Isolation Rating</t>
+  </si>
+  <si>
+    <t>&gt;=1.5</t>
+  </si>
+  <si>
+    <t>kV DC</t>
+  </si>
+  <si>
+    <t>Constraints</t>
+  </si>
+  <si>
+    <t>Formula / Source</t>
+  </si>
+  <si>
+    <t>From Assumptions</t>
+  </si>
+  <si>
+    <t>Bus Nominal Voltage</t>
+  </si>
+  <si>
+    <t>Module Bus Current</t>
+  </si>
+  <si>
+    <t>Operating Point</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Minimum Bus / Minimum Battery</t>
+  </si>
+  <si>
+    <t>Low-voltage edge case</t>
+  </si>
+  <si>
+    <t>Nominal Bus / Nominal Battery</t>
+  </si>
+  <si>
+    <t>Nominal operating point</t>
+  </si>
+  <si>
+    <t>Maximum Bus / Maximum Battery</t>
+  </si>
+  <si>
+    <t>High-voltage edge case</t>
+  </si>
+  <si>
+    <t>Conduction Loss (W)</t>
+  </si>
+  <si>
+    <t>Switching Loss (W)</t>
+  </si>
+  <si>
+    <t>Copper Loss (W)</t>
+  </si>
+  <si>
+    <t>Core Loss (W)</t>
+  </si>
+  <si>
+    <t>Filter Loss (W)</t>
+  </si>
+  <si>
+    <t>Aux Loss (W)</t>
+  </si>
+  <si>
+    <t>Total Loss (W)</t>
+  </si>
+  <si>
+    <t>Requirement</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>25-50% &gt;= 98.5%</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>50-100% &gt;= 99.0%</t>
+  </si>
+  <si>
+    <t>99.21%-99.50%</t>
+  </si>
+  <si>
+    <t>100% &gt;= 99.5%</t>
+  </si>
+  <si>
+    <t>Selected Value</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Transformer Type</t>
+  </si>
+  <si>
+    <t>High-Frequency Isolation Transformer</t>
+  </si>
+  <si>
+    <t>Used in DAB topology</t>
+  </si>
+  <si>
+    <t>Core Material</t>
+  </si>
+  <si>
+    <t>Nanocrystalline</t>
+  </si>
+  <si>
+    <t>Chosen for high efficiency at power scale</t>
+  </si>
+  <si>
+    <t>Tradeoff between size and switching loss</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>Galvanic Isolation + Voltage Matching</t>
+  </si>
+  <si>
+    <t>Required by challenge</t>
+  </si>
+  <si>
+    <t>Estimated Copper Loss</t>
+  </si>
+  <si>
+    <t>From loss budget</t>
+  </si>
+  <si>
+    <t>Estimated Core Loss</t>
+  </si>
+  <si>
+    <t>Total Magnetics Loss</t>
+  </si>
+  <si>
+    <t>Copper + core</t>
+  </si>
+  <si>
+    <t>Turns Ratio (Assumed)</t>
+  </si>
+  <si>
+    <t>Supports 800V to ~1000V nominal conversion</t>
+  </si>
+  <si>
+    <t>Design Note</t>
+  </si>
+  <si>
+    <t>Magnetics losses include copper losses in the windings and core losses due to hysteresis and eddy currents. A nanocrystalline core is assumed to support high-power, high-efficiency operation.</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>Estimated Impact</t>
+  </si>
+  <si>
+    <t>Device Type</t>
+  </si>
+  <si>
+    <t>Lower switching loss than silicon</t>
+  </si>
+  <si>
+    <t>Supports high efficiency</t>
+  </si>
+  <si>
+    <t>Voltage Class</t>
+  </si>
+  <si>
+    <t>Suitable for high-voltage modular converter</t>
+  </si>
+  <si>
+    <t>Improves margin</t>
+  </si>
+  <si>
+    <t>Topology Role</t>
+  </si>
+  <si>
+    <t>Primary/Secondary Bridges</t>
+  </si>
+  <si>
+    <t>Used in DAB switching stages</t>
+  </si>
+  <si>
+    <t>Bidirectional switching</t>
+  </si>
+  <si>
+    <t>Estimated Conduction Loss</t>
+  </si>
+  <si>
+    <t>From system loss budget</t>
+  </si>
+  <si>
+    <t>High-load loss component</t>
+  </si>
+  <si>
+    <t>Estimated Switching Loss</t>
+  </si>
+  <si>
+    <t>Depends on frequency</t>
+  </si>
+  <si>
+    <t>Why Not Silicon IGBT</t>
+  </si>
+  <si>
+    <t>Higher switching losses</t>
+  </si>
+  <si>
+    <t>Less suitable for high-frequency operation</t>
+  </si>
+  <si>
+    <t>Lower efficiency</t>
+  </si>
+  <si>
+    <t>Selection Note</t>
+  </si>
+  <si>
+    <t>SiC MOSFETs were selected for lower switching losses, higher voltage capability, and better efficiency at high power and switching frequency than conventional silicon devices.</t>
+  </si>
+  <si>
+    <t>Challenge condition</t>
+  </si>
+  <si>
+    <t>Semiconductor limit</t>
+  </si>
+  <si>
+    <t>Transformer/core limit</t>
+  </si>
+  <si>
+    <t>Assumed for MW-scale converter</t>
+  </si>
+  <si>
+    <t>Full-Load Loss</t>
+  </si>
+  <si>
+    <t>Must be removed thermally</t>
+  </si>
+  <si>
+    <t>Per-Module Loss</t>
+  </si>
+  <si>
+    <t>For 5 modules</t>
+  </si>
+  <si>
+    <t>Thermal Design Goal</t>
+  </si>
+  <si>
+    <t>Keep all components below limits</t>
+  </si>
+  <si>
+    <t>Concept-level requirement</t>
+  </si>
+  <si>
+    <t>Mode</t>
+  </si>
+  <si>
+    <t>Purpose</t>
+  </si>
+  <si>
+    <t>Where Used</t>
+  </si>
+  <si>
+    <t>CC</t>
+  </si>
+  <si>
+    <t>Constant Current</t>
+  </si>
+  <si>
+    <t>Bulk battery charging</t>
+  </si>
+  <si>
+    <t>Limits current during charge</t>
+  </si>
+  <si>
+    <t>CV</t>
+  </si>
+  <si>
+    <t>Constant Voltage</t>
+  </si>
+  <si>
+    <t>End-of-charge battery control</t>
+  </si>
+  <si>
+    <t>Prevents battery overvoltage</t>
+  </si>
+  <si>
+    <t>CP</t>
+  </si>
+  <si>
+    <t>Constant Power</t>
+  </si>
+  <si>
+    <t>Data center bus support / dispatch</t>
+  </si>
+  <si>
+    <t>Maintains set power exchange</t>
+  </si>
+  <si>
+    <t>Phase Shift Control</t>
+  </si>
+  <si>
+    <t>Power flow control in DAB</t>
+  </si>
+  <si>
+    <t>Both directions</t>
+  </si>
+  <si>
+    <t>Controls magnitude and direction of power</t>
+  </si>
+  <si>
+    <t>Control Note</t>
+  </si>
+  <si>
+    <t>The DAB converter uses phase-shift control to regulate bidirectional power transfer while supporting CC, CV, and CP operating modes required by the challenge.</t>
+  </si>
+  <si>
+    <t>Our Design</t>
+  </si>
+  <si>
+    <t>Bus Voltage Range</t>
+  </si>
+  <si>
+    <t>720-880 V</t>
+  </si>
+  <si>
+    <t>800 V nominal, 720-880 V supported</t>
+  </si>
+  <si>
+    <t>Rated Power</t>
+  </si>
+  <si>
+    <t>2.5 MW bidirectional</t>
+  </si>
+  <si>
+    <t>5 x 500 kW = 2.5 MW</t>
+  </si>
+  <si>
+    <t>Isolation</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>HF transformer in DAB</t>
+  </si>
+  <si>
+    <t>100% Load Efficiency</t>
+  </si>
+  <si>
+    <t>50-100% Efficiency</t>
+  </si>
+  <si>
+    <t>25-50% Efficiency</t>
+  </si>
+  <si>
+    <t>98.74%-99.21%</t>
+  </si>
+  <si>
+    <t>Control Modes</t>
+  </si>
+  <si>
+    <t>CC/CV/CP</t>
+  </si>
+  <si>
+    <t>Included</t>
+  </si>
+  <si>
+    <t>Loss Budget</t>
+  </si>
+  <si>
+    <t>Included by component</t>
+  </si>
+  <si>
+    <t>Magnetics Design</t>
+  </si>
+  <si>
+    <t>Semiconductor Selection</t>
+  </si>
+  <si>
+    <t>Battery Architecture</t>
+  </si>
+  <si>
+    <t>Series-connected HV battery stack</t>
+  </si>
+  <si>
+    <t>Modular Architecture</t>
+  </si>
+  <si>
+    <t>5 x 500 kW DAB modules</t>
+  </si>
+  <si>
+    <t>Max Bus Current</t>
+  </si>
+  <si>
+    <t>Meets challenge insulation target</t>
+  </si>
+  <si>
+    <t>Soft-Switching Relevance</t>
+  </si>
+  <si>
+    <t>Supports lower switching loss</t>
+  </si>
+  <si>
+    <t>Useful for high-efficiency DAB operation</t>
+  </si>
+  <si>
+    <t>Per-Module Power</t>
+  </si>
+  <si>
+    <t>For 5-module architecture</t>
+  </si>
+  <si>
+    <t>Ramp Rate Limit</t>
+  </si>
+  <si>
+    <t>Protects battery health and bus stability</t>
+  </si>
+  <si>
+    <t>Concept-level assumption</t>
+  </si>
+  <si>
+    <t>Bidirectional Full-Range Operation</t>
+  </si>
+  <si>
+    <t>Charge/discharge supported across design range</t>
+  </si>
+  <si>
+    <t>Thermal Constraints</t>
+  </si>
+  <si>
+    <t>Included in Thermal_Constraints tab</t>
+  </si>
+  <si>
+    <t>Fault Handling Definition</t>
+  </si>
+  <si>
+    <t>Concept-level protection strategy to be documented</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Fault Condition</t>
+  </si>
+  <si>
+    <t>Response Strategy</t>
+  </si>
+  <si>
+    <t>Battery short circuit</t>
+  </si>
+  <si>
+    <t>Isolate battery side and shut down converter</t>
+  </si>
+  <si>
+    <t>Bus short upstream</t>
+  </si>
+  <si>
+    <t>Disconnect converter from HVDC bus</t>
+  </si>
+  <si>
+    <t>Battery overvoltage</t>
+  </si>
+  <si>
+    <t>Block charging / enter CV limit</t>
+  </si>
+  <si>
+    <t>Battery undervoltage</t>
+  </si>
+  <si>
+    <t>Block discharge</t>
+  </si>
+  <si>
+    <t>Bus overvoltage</t>
+  </si>
+  <si>
+    <t>Reduce export / shut down if limit exceeded</t>
+  </si>
+  <si>
+    <t>Bus undervoltage</t>
+  </si>
+  <si>
+    <t>Limit charging / support bus if allowed</t>
+  </si>
+  <si>
+    <t>Loss of BMS communication</t>
+  </si>
+  <si>
+    <t>Enter safe shutdown state</t>
+  </si>
+  <si>
+    <t>Overtemperature</t>
+  </si>
+  <si>
+    <t>Reduce power or trip converter</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="172" formatCode="0.0000"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.00000%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -176,8 +820,38 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -196,8 +870,110 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -257,11 +1033,45 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -272,12 +1082,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -287,15 +1102,168 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -732,7 +1700,506 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Converter Efficiency vs Load</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Efficiency!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Efficiency</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="22225" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Efficiency!$A$2:$A$5</c:f>
+              <c:numCache>
+                <c:formatCode>0%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.25</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.75</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Efficiency!$C$2:$C$5</c:f>
+              <c:numCache>
+                <c:formatCode>0.00%</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.98740000000000006</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.99209999999999998</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.99390000000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.995</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FF0D-4BA6-A79C-7FEEF092E498}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="79760944"/>
+        <c:axId val="79767184"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="79760944"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Load</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> %</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="accent1">
+                <a:alpha val="96000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="79767184"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+        <c:majorUnit val="0.1"/>
+        <c:minorUnit val="5.000000000000001E-2"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="79767184"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Efficiency</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="0.00%" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="dk1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="79760944"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="lt1"/>
+    </a:solidFill>
+    <a:ln w="15875" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="95000"/>
+          <a:lumOff val="5000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1288,6 +2755,526 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="241">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200" cap="all"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="50000"/>
+        <a:lumOff val="50000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="22225" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout size="6"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1600" b="1" kern="1200" cap="all" spc="120" normalizeH="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="800" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1309,6 +3296,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BEFF5067-E13C-1CED-7539-9F4D5AB2FBE5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>403860</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>87630</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>944880</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BCDE1554-6F3C-426B-03DF-4A5561961B87}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1657,48 +3685,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="G1" s="14" t="s">
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="G1" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="10"/>
+      <c r="J1" s="10"/>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="8" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="11"/>
-      <c r="B3" s="9" t="s">
+      <c r="A3" s="12"/>
+      <c r="B3" s="8" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="2">
@@ -1723,8 +3751,8 @@
       </c>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="11"/>
-      <c r="B4" s="9" t="s">
+      <c r="A4" s="12"/>
+      <c r="B4" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="2">
@@ -1749,8 +3777,8 @@
       </c>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="11"/>
-      <c r="B5" s="9" t="s">
+      <c r="A5" s="12"/>
+      <c r="B5" s="8" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="2">
@@ -1775,8 +3803,8 @@
       </c>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="12"/>
-      <c r="B6" s="9" t="s">
+      <c r="A6" s="13"/>
+      <c r="B6" s="8" t="s">
         <v>9</v>
       </c>
       <c r="C6" s="2">
@@ -1799,17 +3827,17 @@
       </c>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="8"/>
+      <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="J7" s="3"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="8" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="2">
@@ -1821,8 +3849,8 @@
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="11"/>
-      <c r="B9" s="9" t="s">
+      <c r="A9" s="12"/>
+      <c r="B9" s="8" t="s">
         <v>12</v>
       </c>
       <c r="C9" s="3">
@@ -1834,8 +3862,8 @@
       </c>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="11"/>
-      <c r="B10" s="9" t="s">
+      <c r="A10" s="12"/>
+      <c r="B10" s="8" t="s">
         <v>13</v>
       </c>
       <c r="C10" s="5">
@@ -1847,8 +3875,8 @@
       </c>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="12"/>
-      <c r="B11" s="9" t="s">
+      <c r="A11" s="13"/>
+      <c r="B11" s="8" t="s">
         <v>14</v>
       </c>
       <c r="C11" s="3">
@@ -1860,16 +3888,16 @@
       </c>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="8"/>
+      <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="8" t="s">
         <v>16</v>
       </c>
       <c r="C13" s="2">
@@ -1880,8 +3908,8 @@
       </c>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="11"/>
-      <c r="B14" s="9" t="s">
+      <c r="A14" s="12"/>
+      <c r="B14" s="8" t="s">
         <v>17</v>
       </c>
       <c r="C14" s="2">
@@ -1892,8 +3920,8 @@
       </c>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="11"/>
-      <c r="B15" s="9" t="s">
+      <c r="A15" s="12"/>
+      <c r="B15" s="8" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="2">
@@ -1904,8 +3932,8 @@
       </c>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="11"/>
-      <c r="B16" s="9" t="s">
+      <c r="A16" s="12"/>
+      <c r="B16" s="8" t="s">
         <v>19</v>
       </c>
       <c r="C16" s="2">
@@ -1916,8 +3944,8 @@
       </c>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="11"/>
-      <c r="B17" s="9" t="s">
+      <c r="A17" s="12"/>
+      <c r="B17" s="8" t="s">
         <v>20</v>
       </c>
       <c r="C17" s="2">
@@ -1928,8 +3956,8 @@
       </c>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" s="11"/>
-      <c r="B18" s="9" t="s">
+      <c r="A18" s="12"/>
+      <c r="B18" s="8" t="s">
         <v>21</v>
       </c>
       <c r="C18" s="2">
@@ -1940,8 +3968,8 @@
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="12"/>
-      <c r="B19" s="9" t="s">
+      <c r="A19" s="13"/>
+      <c r="B19" s="8" t="s">
         <v>22</v>
       </c>
       <c r="C19" s="5">
@@ -1978,9 +4006,1835 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E511615-F28A-4614-A88C-F6F99EE54A74}">
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="33.44140625" customWidth="1"/>
+    <col min="2" max="2" width="27.6640625" customWidth="1"/>
+    <col min="3" max="3" width="48.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="22.8" customHeight="1">
+      <c r="A1" s="66" t="s">
+        <v>97</v>
+      </c>
+      <c r="B1" s="53" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="66" t="s">
+        <v>181</v>
+      </c>
+      <c r="D1" s="53" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>183</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>184</v>
+      </c>
+      <c r="D2" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>187</v>
+      </c>
+      <c r="D3" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="32" t="s">
+        <v>188</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>190</v>
+      </c>
+      <c r="D4" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="32" t="s">
+        <v>191</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>64</v>
+      </c>
+      <c r="C5" s="46">
+        <v>0.995</v>
+      </c>
+      <c r="D5" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="D7" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>196</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>197</v>
+      </c>
+      <c r="D8" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>199</v>
+      </c>
+      <c r="D9" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="32" t="s">
+        <v>200</v>
+      </c>
+      <c r="B10" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>197</v>
+      </c>
+      <c r="D10" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="32" t="s">
+        <v>201</v>
+      </c>
+      <c r="B11" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>197</v>
+      </c>
+      <c r="D11" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="32" t="s">
+        <v>216</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>217</v>
+      </c>
+      <c r="D12" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="32" t="s">
+        <v>218</v>
+      </c>
+      <c r="B13" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="C13" s="31" t="s">
+        <v>219</v>
+      </c>
+      <c r="D13" s="67" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="32" t="s">
+        <v>220</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>189</v>
+      </c>
+      <c r="C14" s="31" t="s">
+        <v>221</v>
+      </c>
+      <c r="D14" s="47" t="s">
+        <v>222</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{38FDFBA1-9F2C-4188-9097-91243CFDB78D}">
+  <dimension ref="A1:B9"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="26.44140625" customWidth="1"/>
+    <col min="2" max="2" width="43.6640625" customWidth="1"/>
+    <col min="3" max="3" width="18.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="27" customHeight="1">
+      <c r="A1" s="52" t="s">
+        <v>223</v>
+      </c>
+      <c r="B1" s="52" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="27" customHeight="1">
+      <c r="A2" s="71" t="s">
+        <v>225</v>
+      </c>
+      <c r="B2" s="70" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="27" customHeight="1">
+      <c r="A3" s="71" t="s">
+        <v>227</v>
+      </c>
+      <c r="B3" s="70" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="27" customHeight="1">
+      <c r="A4" s="71" t="s">
+        <v>229</v>
+      </c>
+      <c r="B4" s="70" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="27" customHeight="1">
+      <c r="A5" s="71" t="s">
+        <v>231</v>
+      </c>
+      <c r="B5" s="70" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="27" customHeight="1">
+      <c r="A6" s="71" t="s">
+        <v>233</v>
+      </c>
+      <c r="B6" s="70" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="27" customHeight="1">
+      <c r="A7" s="71" t="s">
+        <v>235</v>
+      </c>
+      <c r="B7" s="70" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="27" customHeight="1">
+      <c r="A8" s="71" t="s">
+        <v>237</v>
+      </c>
+      <c r="B8" s="70" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="27" customHeight="1">
+      <c r="A9" s="71" t="s">
+        <v>239</v>
+      </c>
+      <c r="B9" s="70" t="s">
+        <v>240</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{498F749A-658C-41D5-842C-5799910B7650}">
+  <dimension ref="A1:L18"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="13.21875" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" customWidth="1"/>
+    <col min="3" max="3" width="32.77734375" customWidth="1"/>
+    <col min="6" max="6" width="27" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="8.33203125" customWidth="1"/>
+    <col min="11" max="11" width="20.21875" customWidth="1"/>
+    <col min="12" max="12" width="31.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A1" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="22"/>
+      <c r="F1" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="G1" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="I1" s="21" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A2" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="23" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="24">
+        <v>800</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="33" t="s">
+        <v>63</v>
+      </c>
+      <c r="G2" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2" s="24">
+        <v>99.5</v>
+      </c>
+      <c r="I2" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="K2" s="68" t="s">
+        <v>202</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A3" s="16"/>
+      <c r="B3" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="24">
+        <v>720</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="33" t="s">
+        <v>66</v>
+      </c>
+      <c r="G3" s="34" t="s">
+        <v>67</v>
+      </c>
+      <c r="H3" s="24">
+        <v>99</v>
+      </c>
+      <c r="I3" s="35" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="68" t="s">
+        <v>204</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A4" s="16"/>
+      <c r="B4" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="24">
+        <v>880</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="G4" s="34" t="s">
+        <v>69</v>
+      </c>
+      <c r="H4" s="24">
+        <v>98.5</v>
+      </c>
+      <c r="I4" s="35" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A5" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="26">
+        <v>1000</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="33" t="s">
+        <v>70</v>
+      </c>
+      <c r="G5" s="34" t="s">
+        <v>71</v>
+      </c>
+      <c r="H5" s="24">
+        <v>125</v>
+      </c>
+      <c r="I5" s="35" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A6" s="17"/>
+      <c r="B6" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="26">
+        <v>900</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="33" t="s">
+        <v>72</v>
+      </c>
+      <c r="G6" s="34" t="s">
+        <v>73</v>
+      </c>
+      <c r="H6" s="24">
+        <v>120</v>
+      </c>
+      <c r="I6" s="35" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A7" s="17"/>
+      <c r="B7" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="26">
+        <v>1100</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="33" t="s">
+        <v>74</v>
+      </c>
+      <c r="G7" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="H7" s="24">
+        <v>1.5</v>
+      </c>
+      <c r="I7" s="35" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A8" s="17"/>
+      <c r="B8" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="26">
+        <v>10</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A9" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="28">
+        <v>2500000</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A10" s="18"/>
+      <c r="B10" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" s="28">
+        <v>5</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A11" s="18"/>
+      <c r="B11" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" s="28">
+        <v>500000</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A12" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="29" t="s">
+        <v>46</v>
+      </c>
+      <c r="C12" s="30" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A13" s="19"/>
+      <c r="B13" s="29" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A14" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="31" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" s="32" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A15" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="31" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="32">
+        <v>20000</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="32" t="s">
+        <v>206</v>
+      </c>
+      <c r="G15" s="31">
+        <v>3125</v>
+      </c>
+      <c r="H15" s="31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="18.600000000000001" customHeight="1">
+      <c r="A16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A17" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" s="31" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" s="32">
+        <v>40</v>
+      </c>
+      <c r="D17" s="31" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="B18" s="32"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A8"/>
+    <mergeCell ref="A9:A11"/>
+    <mergeCell ref="A12:A13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63342D0E-C6E6-45FA-9A15-F446DF8E54D8}">
+  <dimension ref="A1:D17"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="27.21875" customWidth="1"/>
+    <col min="2" max="2" width="25.33203125" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="24.6" customHeight="1">
+      <c r="A1" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C1" s="38" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="38" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A2" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="31">
+        <v>2500000</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A3" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="31">
+        <v>800</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A4" s="32" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="31">
+        <v>1000</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A5" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="31">
+        <v>5</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A6" s="32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="31">
+        <f>C2/C3</f>
+        <v>3125</v>
+      </c>
+      <c r="C6" s="31">
+        <v>3125</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A7" s="32" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="31">
+        <f>C2/C4</f>
+        <v>2500</v>
+      </c>
+      <c r="C7" s="31">
+        <v>2500</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A8" s="32" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="31">
+        <f>C2/C5</f>
+        <v>500000</v>
+      </c>
+      <c r="C8" s="31">
+        <v>500000</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A9" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9" s="31">
+        <f>C8/C3</f>
+        <v>625</v>
+      </c>
+      <c r="C9" s="31">
+        <v>625</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+    </row>
+    <row r="11" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A11" s="14"/>
+      <c r="B11" s="14"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="14"/>
+    </row>
+    <row r="12" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A12" s="14"/>
+      <c r="B12" s="14"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+    </row>
+    <row r="13" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+    </row>
+    <row r="14" spans="1:4" ht="25.8" customHeight="1">
+      <c r="A14" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A15" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="31">
+        <v>720</v>
+      </c>
+      <c r="C15" s="31">
+        <v>900</v>
+      </c>
+      <c r="D15" s="31" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A16" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="31">
+        <v>800</v>
+      </c>
+      <c r="C16" s="31">
+        <v>1000</v>
+      </c>
+      <c r="D16" s="31" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="18.600000000000001" customHeight="1">
+      <c r="A17" s="31" t="s">
+        <v>88</v>
+      </c>
+      <c r="B17" s="31">
+        <v>880</v>
+      </c>
+      <c r="C17" s="31">
+        <v>1100</v>
+      </c>
+      <c r="D17" s="31" t="s">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D186E9E-38F5-41E5-B016-D9B6DD368117}">
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="21.44140625" customWidth="1"/>
+    <col min="4" max="4" width="19.44140625" customWidth="1"/>
+    <col min="5" max="5" width="16.109375" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" customWidth="1"/>
+    <col min="8" max="8" width="15.109375" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" customWidth="1"/>
+    <col min="10" max="12" width="12.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="24.6" customHeight="1">
+      <c r="A1" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="40" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="40" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="F1" s="40" t="s">
+        <v>93</v>
+      </c>
+      <c r="G1" s="40" t="s">
+        <v>94</v>
+      </c>
+      <c r="H1" s="40" t="s">
+        <v>95</v>
+      </c>
+      <c r="I1" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1" s="39"/>
+      <c r="K1" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" s="40" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" ht="19.8" customHeight="1">
+      <c r="A2" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="B2" s="31">
+        <v>625000</v>
+      </c>
+      <c r="C2" s="31">
+        <v>2200</v>
+      </c>
+      <c r="D2" s="31">
+        <v>1200</v>
+      </c>
+      <c r="E2" s="31">
+        <v>1300</v>
+      </c>
+      <c r="F2" s="31">
+        <v>900</v>
+      </c>
+      <c r="G2" s="31">
+        <v>900</v>
+      </c>
+      <c r="H2" s="31">
+        <v>1500</v>
+      </c>
+      <c r="I2" s="31">
+        <f>SUM(C2:H2)</f>
+        <v>8000</v>
+      </c>
+      <c r="K2" s="41">
+        <v>0.25</v>
+      </c>
+      <c r="L2" s="69">
+        <f>B2/(B2+I2)</f>
+        <v>0.9873617693522907</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="19.8" customHeight="1">
+      <c r="A3" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="B3" s="31">
+        <v>1250000</v>
+      </c>
+      <c r="C3" s="31">
+        <v>3000</v>
+      </c>
+      <c r="D3" s="31">
+        <v>1800</v>
+      </c>
+      <c r="E3" s="31">
+        <v>1700</v>
+      </c>
+      <c r="F3" s="31">
+        <v>1000</v>
+      </c>
+      <c r="G3" s="31">
+        <v>950</v>
+      </c>
+      <c r="H3" s="31">
+        <v>1550</v>
+      </c>
+      <c r="I3" s="31">
+        <f>SUM(C3:H3)</f>
+        <v>10000</v>
+      </c>
+      <c r="K3" s="41">
+        <v>0.5</v>
+      </c>
+      <c r="L3" s="69">
+        <f>B3/(B3+I3)</f>
+        <v>0.99206349206349209</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="19.8" customHeight="1">
+      <c r="A4" s="41">
+        <v>0.75</v>
+      </c>
+      <c r="B4" s="31">
+        <v>1875000</v>
+      </c>
+      <c r="C4" s="31">
+        <v>3600</v>
+      </c>
+      <c r="D4" s="31">
+        <v>2200</v>
+      </c>
+      <c r="E4" s="31">
+        <v>1900</v>
+      </c>
+      <c r="F4" s="31">
+        <v>1100</v>
+      </c>
+      <c r="G4" s="31">
+        <v>1000</v>
+      </c>
+      <c r="H4" s="31">
+        <v>1700</v>
+      </c>
+      <c r="I4" s="31">
+        <f>SUM(C4:H4)</f>
+        <v>11500</v>
+      </c>
+      <c r="K4" s="41">
+        <v>0.75</v>
+      </c>
+      <c r="L4" s="69">
+        <f>B4/(B4+I4)</f>
+        <v>0.99390405512854496</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="19.8" customHeight="1">
+      <c r="A5" s="41">
+        <v>1</v>
+      </c>
+      <c r="B5" s="31">
+        <v>2500000</v>
+      </c>
+      <c r="C5" s="31">
+        <v>4000</v>
+      </c>
+      <c r="D5" s="31">
+        <v>2500</v>
+      </c>
+      <c r="E5" s="31">
+        <v>2000</v>
+      </c>
+      <c r="F5" s="31">
+        <v>1200</v>
+      </c>
+      <c r="G5" s="31">
+        <v>1000</v>
+      </c>
+      <c r="H5" s="31">
+        <v>1800</v>
+      </c>
+      <c r="I5" s="31">
+        <f>SUM(C5:H5)</f>
+        <v>12500</v>
+      </c>
+      <c r="K5" s="41">
+        <v>1</v>
+      </c>
+      <c r="L5" s="69">
+        <f>B5/(B5+I5)</f>
+        <v>0.99502487562189057</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35129CE8-BB74-4EFA-8E82-F13D000CDA16}">
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" customWidth="1"/>
+    <col min="9" max="9" width="19.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="19.8" customHeight="1">
+      <c r="A1" s="44" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="45" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="44" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="I1" s="50" t="s">
+        <v>98</v>
+      </c>
+      <c r="J1" s="49" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A2" s="42">
+        <v>0.25</v>
+      </c>
+      <c r="B2" s="36">
+        <v>8000</v>
+      </c>
+      <c r="C2" s="43">
+        <v>0.98740000000000006</v>
+      </c>
+      <c r="H2" s="31" t="s">
+        <v>100</v>
+      </c>
+      <c r="I2" s="46">
+        <v>0.98740000000000006</v>
+      </c>
+      <c r="J2" s="48" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A3" s="42">
+        <v>0.5</v>
+      </c>
+      <c r="B3" s="36">
+        <v>10000</v>
+      </c>
+      <c r="C3" s="43">
+        <v>0.99209999999999998</v>
+      </c>
+      <c r="H3" s="31" t="s">
+        <v>102</v>
+      </c>
+      <c r="I3" s="31" t="s">
+        <v>103</v>
+      </c>
+      <c r="J3" s="48" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A4" s="42">
+        <v>0.75</v>
+      </c>
+      <c r="B4" s="36">
+        <v>11500</v>
+      </c>
+      <c r="C4" s="43">
+        <v>0.99390000000000001</v>
+      </c>
+      <c r="H4" s="31" t="s">
+        <v>104</v>
+      </c>
+      <c r="I4" s="46">
+        <v>0.995</v>
+      </c>
+      <c r="J4" s="48" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="19.2" customHeight="1">
+      <c r="A5" s="42">
+        <v>1</v>
+      </c>
+      <c r="B5" s="36">
+        <v>12500</v>
+      </c>
+      <c r="C5" s="43">
+        <v>0.995</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A0E95AF-269C-4259-BD38-E1CD066525FB}">
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="22.77734375" customWidth="1"/>
+    <col min="2" max="2" width="34.21875" customWidth="1"/>
+    <col min="4" max="4" width="43.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A1" s="53" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A2" s="51" t="s">
+        <v>107</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A3" s="51" t="s">
+        <v>110</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A4" s="51" t="s">
+        <v>54</v>
+      </c>
+      <c r="B4" s="31">
+        <v>20000</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A5" s="51" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>115</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A6" s="51" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" s="31">
+        <v>2000</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A7" s="51" t="s">
+        <v>119</v>
+      </c>
+      <c r="B7" s="31">
+        <v>1200</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A8" s="51" t="s">
+        <v>120</v>
+      </c>
+      <c r="B8" s="31">
+        <v>3200</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="20.399999999999999" customHeight="1">
+      <c r="A9" s="51" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" s="31">
+        <v>1.25</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="18.600000000000001" customHeight="1">
+      <c r="A10" s="51" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="31">
+        <v>1.5</v>
+      </c>
+      <c r="C10" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="D10" s="31" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="18">
+      <c r="A12" s="57" t="s">
+        <v>124</v>
+      </c>
+      <c r="B12" s="54"/>
+      <c r="C12" s="15"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+    </row>
+    <row r="13" spans="1:9" ht="31.8" customHeight="1">
+      <c r="A13" s="55" t="s">
+        <v>125</v>
+      </c>
+      <c r="B13" s="56"/>
+      <c r="C13" s="56"/>
+      <c r="D13" s="56"/>
+      <c r="E13" s="56"/>
+      <c r="F13" s="56"/>
+      <c r="G13" s="56"/>
+      <c r="H13" s="56"/>
+      <c r="I13" s="56"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:I13"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5CCBAF3-F235-434E-AE49-4A1B6E0F5B1A}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="25.6640625" customWidth="1"/>
+    <col min="4" max="4" width="36.6640625" customWidth="1"/>
+    <col min="5" max="5" width="22.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="36" customHeight="1">
+      <c r="A1" s="58" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="50" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="58" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="50" t="s">
+        <v>126</v>
+      </c>
+      <c r="E1" s="58" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="19.8" customHeight="1">
+      <c r="A2" s="32" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="E2" s="31" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="19.8" customHeight="1">
+      <c r="A3" s="32" t="s">
+        <v>131</v>
+      </c>
+      <c r="B3" s="31">
+        <v>1700</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="E3" s="31" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="19.8" customHeight="1">
+      <c r="A4" s="32" t="s">
+        <v>134</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>136</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="19.8" customHeight="1">
+      <c r="A5" s="32" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="31">
+        <v>4000</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="31" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="19.8" customHeight="1">
+      <c r="A6" s="32" t="s">
+        <v>141</v>
+      </c>
+      <c r="B6" s="31">
+        <v>2500</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>139</v>
+      </c>
+      <c r="E6" s="31" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="19.8" customHeight="1">
+      <c r="A7" s="32" t="s">
+        <v>143</v>
+      </c>
+      <c r="B7" s="31" t="s">
+        <v>144</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>145</v>
+      </c>
+      <c r="E7" s="31" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="17.399999999999999" customHeight="1">
+      <c r="A8" s="32" t="s">
+        <v>208</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>209</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="21.6" customHeight="1">
+      <c r="A11" s="59" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="60" t="s">
+        <v>148</v>
+      </c>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
+      <c r="E12" s="60"/>
+      <c r="F12" s="60"/>
+      <c r="G12" s="60"/>
+      <c r="H12" s="60"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A12:H12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CE81921-1906-4362-9CB4-4826E5DBCB07}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="25.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.21875" customWidth="1"/>
+    <col min="4" max="4" width="29.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="24" customHeight="1">
+      <c r="A1" s="61" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" s="62" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="61" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" s="62" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="24" customHeight="1">
+      <c r="A2" s="32" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="31">
+        <v>40</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="24" customHeight="1">
+      <c r="A3" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="B3" s="31">
+        <v>125</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="24" customHeight="1">
+      <c r="A4" s="32" t="s">
+        <v>72</v>
+      </c>
+      <c r="B4" s="31">
+        <v>120</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="24" customHeight="1">
+      <c r="A5" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="24" customHeight="1">
+      <c r="A6" s="32" t="s">
+        <v>153</v>
+      </c>
+      <c r="B6" s="31">
+        <v>12500</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="31" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="24" customHeight="1">
+      <c r="A7" s="32" t="s">
+        <v>155</v>
+      </c>
+      <c r="B7" s="31">
+        <v>2500</v>
+      </c>
+      <c r="C7" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="24" customHeight="1">
+      <c r="A8" s="32" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="31" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="23.4" customHeight="1">
+      <c r="A9" s="32" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="31">
+        <v>500000</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>5</v>
+      </c>
+      <c r="D9" s="31" t="s">
+        <v>212</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{065E4448-78D4-4DE0-AC6A-FD227B607690}">
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="21.77734375" customWidth="1"/>
+    <col min="2" max="2" width="36.5546875" customWidth="1"/>
+    <col min="3" max="3" width="29.44140625" customWidth="1"/>
+    <col min="4" max="4" width="35.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="21.6" customHeight="1">
+      <c r="A1" s="63" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="63" t="s">
+        <v>161</v>
+      </c>
+      <c r="C1" s="63" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" s="63" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="21.6" customHeight="1">
+      <c r="A2" s="32" t="s">
+        <v>163</v>
+      </c>
+      <c r="B2" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="C2" s="31" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="21.6" customHeight="1">
+      <c r="A3" s="32" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="31" t="s">
+        <v>168</v>
+      </c>
+      <c r="C3" s="31" t="s">
+        <v>169</v>
+      </c>
+      <c r="D3" s="31" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="21.6" customHeight="1">
+      <c r="A4" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="B4" s="31" t="s">
+        <v>172</v>
+      </c>
+      <c r="C4" s="31" t="s">
+        <v>173</v>
+      </c>
+      <c r="D4" s="31" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="21.6" customHeight="1">
+      <c r="A5" s="32" t="s">
+        <v>175</v>
+      </c>
+      <c r="B5" s="31" t="s">
+        <v>176</v>
+      </c>
+      <c r="C5" s="31" t="s">
+        <v>177</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="20.399999999999999" customHeight="1">
+      <c r="A6" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="B6" s="31" t="s">
+        <v>214</v>
+      </c>
+      <c r="C6" s="31" t="s">
+        <v>215</v>
+      </c>
+      <c r="D6" s="31"/>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="65" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="64" t="s">
+        <v>180</v>
+      </c>
+      <c r="B10" s="64"/>
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A10:F10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010012AE384354536C4787A8543A0DFBB11B" ma:contentTypeVersion="6" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3bc2b737abf995cd71d95abe1e4782a1">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="301349ed-c51a-435a-8255-5a878db350e9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fa0a8f3fca150e90200a4a989577875e" ns3:_="">
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="301349ed-c51a-435a-8255-5a878db350e9" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010012AE384354536C4787A8543A0DFBB11B" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1022a0dc21405b74310b87ae03793539">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="301349ed-c51a-435a-8255-5a878db350e9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dc610f19cbafaf7828a25c7e06ac6bf6" ns3:_="">
     <xsd:import namespace="301349ed-c51a-435a-8255-5a878db350e9"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -1994,6 +5848,10 @@
                 <xsd:element ref="ns3:MediaServiceSearchProperties" minOccurs="0"/>
                 <xsd:element ref="ns3:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns3:_activity" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceSystemTags" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns3:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -2032,6 +5890,28 @@
     <xsd:element name="_activity" ma:index="13" nillable="true" ma:displayName="_activity" ma:hidden="true" ma:internalName="_activity">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSystemTags" ma:index="14" nillable="true" ma:displayName="MediaServiceSystemTags" ma:hidden="true" ma:internalName="MediaServiceSystemTags" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -2134,25 +6014,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76641656-DAF8-409B-892B-012B16E2B7F3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="301349ed-c51a-435a-8255-5a878db350e9" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCBFD1E0-67B7-469A-BD7D-D863E2DCDC15}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="301349ed-c51a-435a-8255-5a878db350e9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C257039-E6E8-469A-848D-7A21CC3178C0}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C511FE14-63E2-4152-9A79-511E8EE9E625}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -2167,28 +6054,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76641656-DAF8-409B-892B-012B16E2B7F3}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BCBFD1E0-67B7-469A-BD7D-D863E2DCDC15}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="301349ed-c51a-435a-8255-5a878db350e9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>